<commit_message>
Update wedstrijddata - 14 oktober 2026
</commit_message>
<xml_diff>
--- a/Driebanden moyenne.xlsx
+++ b/Driebanden moyenne.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\MyTech\Github\biljart\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tenneteu-my.sharepoint.com/personal/sandjai_ramasray_tennet_eu/Documents/GithubCopilotWS/Biljart/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBDBB7B6-5F1A-433D-9CCB-24CD5CBE0AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4EB315A-5565-4A70-9642-A2FD8F8E455C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="1425" windowWidth="20130" windowHeight="20175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="795" yWindow="795" windowWidth="33105" windowHeight="19110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -51,16 +51,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -76,7 +68,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -84,31 +76,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Total" xfId="1" builtinId="25"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -123,10 +102,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -164,7 +147,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -270,7 +253,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -412,7 +395,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -420,29 +403,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46073</v>
       </c>
@@ -636,57 +618,45 @@
         <v>46108</v>
       </c>
       <c r="B12">
-        <f>7/25</f>
         <v>0.28000000000000003</v>
       </c>
       <c r="C12">
-        <f>5/26</f>
         <v>0.19230769230769232</v>
       </c>
       <c r="D12">
-        <f>10/25</f>
         <v>0.4</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13">
-        <f>7/25</f>
         <v>0.28000000000000003</v>
       </c>
       <c r="C13">
-        <f>7/25</f>
         <v>0.28000000000000003</v>
       </c>
       <c r="D13">
-        <f>7/25</f>
         <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14">
-        <f>13/30</f>
         <v>0.43333333333333335</v>
       </c>
       <c r="C14">
-        <f>7/30</f>
         <v>0.23333333333333334</v>
       </c>
       <c r="D14">
-        <f>15/30</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15">
-        <f>10/30</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="C15">
-        <f>18/30</f>
         <v>0.6</v>
       </c>
       <c r="D15">
-        <f>7/30</f>
         <v>0.23333333333333334</v>
       </c>
     </row>
@@ -695,55 +665,43 @@
         <v>46115</v>
       </c>
       <c r="B16">
-        <f>10/30</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="C16">
-        <f>9/30</f>
         <v>0.3</v>
       </c>
       <c r="D16">
-        <f>7/30</f>
         <v>0.23333333333333334</v>
       </c>
       <c r="E16">
-        <f>21/30</f>
         <v>0.7</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17">
-        <f>10/30</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="C17">
-        <f>7/30</f>
         <v>0.23333333333333334</v>
       </c>
       <c r="D17">
-        <f>6/30</f>
         <v>0.2</v>
       </c>
       <c r="E17">
-        <f>17/30</f>
         <v>0.56666666666666665</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B18">
-        <f>12/30</f>
         <v>0.4</v>
       </c>
       <c r="C18">
-        <f>5/30</f>
         <v>0.16666666666666666</v>
       </c>
       <c r="D18">
-        <f>10/30</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="E18">
-        <f>12/30</f>
         <v>0.4</v>
       </c>
     </row>
@@ -804,7 +762,188 @@
         <v>0.3</v>
       </c>
     </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>46129</v>
+      </c>
+      <c r="B22">
+        <f>2/30</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="C22" s="2">
+        <f>8/30</f>
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="D22">
+        <f>7/30</f>
+        <v>0.23333333333333334</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <f>10/30</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C23">
+        <f>11/30</f>
+        <v>0.36666666666666664</v>
+      </c>
+      <c r="D23">
+        <f>11/30</f>
+        <v>0.36666666666666664</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <f>12/30</f>
+        <v>0.4</v>
+      </c>
+      <c r="C24">
+        <f>12/30</f>
+        <v>0.4</v>
+      </c>
+      <c r="D24">
+        <f>8/30</f>
+        <v>0.26666666666666666</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>46136</v>
+      </c>
+      <c r="B25">
+        <f>16/30</f>
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="C25">
+        <f>14/30</f>
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="D25">
+        <f>7/30</f>
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="E25">
+        <f>16/30</f>
+        <v>0.53333333333333333</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B26">
+        <f>10/30</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C26">
+        <f>14/30</f>
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="D26">
+        <f>4/39</f>
+        <v>0.10256410256410256</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B27">
+        <f>10/30</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C27">
+        <f>9/30</f>
+        <v>0.3</v>
+      </c>
+      <c r="D27">
+        <f>6/30</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>46151</v>
+      </c>
+      <c r="B28" s="3">
+        <f>7/30</f>
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="C28">
+        <f>19/30</f>
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="D28">
+        <f>4/30</f>
+        <v>0.13333333333333333</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <f>8/30</f>
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="C29">
+        <f>10/30</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D29">
+        <f>6/30</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <f>9/25</f>
+        <v>0.36</v>
+      </c>
+      <c r="C30">
+        <f>14/25</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="D30">
+        <f>12/25</f>
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>46241</v>
+      </c>
+      <c r="B32">
+        <f>9/30</f>
+        <v>0.3</v>
+      </c>
+      <c r="C32">
+        <f>13/30</f>
+        <v>0.43333333333333335</v>
+      </c>
+      <c r="D32">
+        <f>14/30</f>
+        <v>0.46666666666666667</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <f>14/30</f>
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="C33">
+        <f>14/30</f>
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="D33">
+        <f>9/30</f>
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>46248</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{6e118e09-08be-4360-a815-3fc29828016d}" enabled="1" method="Standard" siteId="{15b734ef-4a07-47e7-90f4-22cc84a7af23}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>